<commit_message>
Desk build: onepager_draft AGI
</commit_message>
<xml_diff>
--- a/models/AGI/2026-10-27_AGI_Model_v2026Q2.xlsx
+++ b/models/AGI/2026-10-27_AGI_Model_v2026Q2.xlsx
@@ -1686,7 +1686,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
@@ -1917,7 +1917,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
@@ -1980,7 +1980,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K53"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
@@ -2847,7 +2847,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
@@ -3793,7 +3793,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E81"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
@@ -4660,7 +4660,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z18"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
@@ -5648,7 +5648,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="12"/>
@@ -5969,7 +5969,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
@@ -6227,7 +6227,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
@@ -6370,7 +6370,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>

</xml_diff>